<commit_message>
Itog table: discounts filled, totals label placement
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/ITOG_LOTS_1410.xlsx
+++ b/ITOG_LOTS_1410.xlsx
@@ -909,7 +909,9 @@
       <c r="K6" s="8" t="n">
         <v>2177384</v>
       </c>
-      <c r="L6" s="10" t="n"/>
+      <c r="L6" s="10" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M6" s="11" t="n">
         <v>1478527</v>
       </c>
@@ -1069,7 +1071,9 @@
       <c r="K8" s="8" t="n">
         <v>714880</v>
       </c>
-      <c r="L8" s="10" t="n"/>
+      <c r="L8" s="10" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M8" s="11" t="n">
         <v>449028</v>
       </c>
@@ -1229,7 +1233,9 @@
       <c r="K10" s="8" t="n">
         <v>1630827</v>
       </c>
-      <c r="L10" s="10" t="n"/>
+      <c r="L10" s="10" t="n">
+        <v>0.17</v>
+      </c>
       <c r="M10" s="11" t="n">
         <v>323274</v>
       </c>
@@ -1470,7 +1476,9 @@
       <c r="K13" s="8" t="n">
         <v>609645</v>
       </c>
-      <c r="L13" s="10" t="n"/>
+      <c r="L13" s="10" t="n">
+        <v>0.14</v>
+      </c>
       <c r="M13" s="13" t="n">
         <v>247436</v>
       </c>
@@ -1630,7 +1638,9 @@
       <c r="K15" s="8" t="n">
         <v>266390</v>
       </c>
-      <c r="L15" s="10" t="n"/>
+      <c r="L15" s="10" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M15" s="13" t="n">
         <v>189886</v>
       </c>
@@ -2025,7 +2035,9 @@
       <c r="I20" s="8" t="n"/>
       <c r="J20" s="10" t="n"/>
       <c r="K20" s="8" t="n"/>
-      <c r="L20" s="10" t="n"/>
+      <c r="L20" s="10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
       <c r="M20" s="13" t="n">
         <v>116467</v>
       </c>
@@ -2175,7 +2187,9 @@
       <c r="I22" s="8" t="n"/>
       <c r="J22" s="10" t="n"/>
       <c r="K22" s="8" t="n"/>
-      <c r="L22" s="10" t="n"/>
+      <c r="L22" s="10" t="n">
+        <v>0.07000000000000001</v>
+      </c>
       <c r="M22" s="13" t="n">
         <v>99875</v>
       </c>
@@ -2414,7 +2428,9 @@
       <c r="K25" s="8" t="n">
         <v>153372359</v>
       </c>
-      <c r="L25" s="10" t="n"/>
+      <c r="L25" s="10" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M25" s="11" t="n">
         <v>39758366</v>
       </c>
@@ -2493,7 +2509,9 @@
       <c r="K26" s="8" t="n">
         <v>66162726</v>
       </c>
-      <c r="L26" s="10" t="n"/>
+      <c r="L26" s="10" t="n">
+        <v>0.1</v>
+      </c>
       <c r="M26" s="11" t="n">
         <v>32511680</v>
       </c>
@@ -2528,14 +2546,14 @@
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="17" t="inlineStr"/>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>ИТОГО — обычные условия</t>
-        </is>
-      </c>
+      <c r="B27" s="17" t="inlineStr"/>
       <c r="C27" s="17" t="inlineStr"/>
       <c r="D27" s="17" t="inlineStr"/>
-      <c r="E27" s="17" t="inlineStr"/>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>ИТОГО — обычные условия</t>
+        </is>
+      </c>
       <c r="F27" s="17" t="inlineStr"/>
       <c r="G27" s="17" t="inlineStr"/>
       <c r="H27" s="18" t="n">
@@ -2563,14 +2581,14 @@
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="17" t="inlineStr"/>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>ИТОГО — с крупными (жёсткие условия)</t>
-        </is>
-      </c>
+      <c r="B28" s="17" t="inlineStr"/>
       <c r="C28" s="17" t="inlineStr"/>
       <c r="D28" s="17" t="inlineStr"/>
-      <c r="E28" s="17" t="inlineStr"/>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>ИТОГО — с крупными (жёсткие условия)</t>
+        </is>
+      </c>
       <c r="F28" s="17" t="inlineStr"/>
       <c r="G28" s="17" t="inlineStr"/>
       <c r="H28" s="18" t="n">

</xml_diff>

<commit_message>
Itog: add price source links per position
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/ITOG_LOTS_1410.xlsx
+++ b/ITOG_LOTS_1410.xlsx
@@ -102,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -148,6 +148,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -532,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R105"/>
+  <dimension ref="A1:T105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -552,7 +555,9 @@
     <col width="15" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="55" customWidth="1" min="18" max="18"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -578,6 +583,8 @@
       <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
       <c r="R1" s="2" t="n"/>
+      <c r="S1" s="2" t="n"/>
+      <c r="T1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -602,6 +609,8 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
     </row>
     <row r="3" ht="51" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -692,6 +701,16 @@
       <c r="R3" s="3" t="inlineStr">
         <is>
           <t>Откуда себестоимость</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Где цена (ссылка)</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Ещё источники</t>
         </is>
       </c>
     </row>
@@ -766,6 +785,18 @@
           <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410)</t>
         </is>
       </c>
+      <c r="S4" s="7" t="inlineStr">
+        <is>
+          <t>esolk.ru</t>
+        </is>
+      </c>
+      <c r="T4" s="8" t="inlineStr">
+        <is>
+          <t>https://nsmgr.ru/reagenty/tekhnicheskaya-sol/big-begi
+https://sknerud.ru/reagent/sol-texnicheskaya/
+https://vektor-e.ru/sol/</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -836,6 +867,18 @@
       <c r="R5" s="8" t="inlineStr">
         <is>
           <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410)</t>
+        </is>
+      </c>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>esolk.ru</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
+        <is>
+          <t>https://nsmgr.ru/reagenty/tekhnicheskaya-sol/big-begi
+https://sknerud.ru/reagent/sol-texnicheskaya/
+https://vektor-e.ru/sol/</t>
         </is>
       </c>
     </row>
@@ -898,6 +941,8 @@
           <t>по позициям ниже</t>
         </is>
       </c>
+      <c r="S6" s="4" t="n"/>
+      <c r="T6" s="4" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr"/>
@@ -942,6 +987,17 @@
           <t>справочник: Жилет сигнальный</t>
         </is>
       </c>
+      <c r="S7" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T7" s="13" t="inlineStr">
+        <is>
+          <t>https://www.trakt.ru/product/138206/
+https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="13" t="inlineStr"/>
@@ -986,6 +1042,17 @@
           <t>справочник: Жилет утепленный</t>
         </is>
       </c>
+      <c r="S8" s="16" t="inlineStr">
+        <is>
+          <t>ivuniforma.ru</t>
+        </is>
+      </c>
+      <c r="T8" s="13" t="inlineStr">
+        <is>
+          <t>https://www.trakt.ru/product/12021/
+https://www.spets.ru/products/spetsodezhda/odezhda_dlya_okhrannykh_struktur/</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="13" t="inlineStr"/>
@@ -1030,6 +1097,16 @@
           <t>Фабрикант 975 / Ивсотекс 1 250</t>
         </is>
       </c>
+      <c r="S9" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T9" s="13" t="inlineStr">
+        <is>
+          <t>https://ivsoteks.ru/specodejda</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="13" t="inlineStr"/>
@@ -1074,6 +1151,17 @@
           <t>справочник: Костюм летний рабочий</t>
         </is>
       </c>
+      <c r="S10" s="16" t="inlineStr">
+        <is>
+          <t>ivuniforma.ru</t>
+        </is>
+      </c>
+      <c r="T10" s="13" t="inlineStr">
+        <is>
+          <t>https://ivsoteks.ru/specodejda
+https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="13" t="inlineStr"/>
@@ -1118,6 +1206,17 @@
           <t>справочник: Костюм летний рабочий</t>
         </is>
       </c>
+      <c r="S11" s="16" t="inlineStr">
+        <is>
+          <t>ivuniforma.ru</t>
+        </is>
+      </c>
+      <c r="T11" s="13" t="inlineStr">
+        <is>
+          <t>https://ivsoteks.ru/specodejda
+https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="13" t="inlineStr"/>
@@ -1162,6 +1261,17 @@
           <t>справочник: Куртка утепленная</t>
         </is>
       </c>
+      <c r="S12" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T12" s="13" t="inlineStr">
+        <is>
+          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
+https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="13" t="inlineStr"/>
@@ -1206,6 +1316,17 @@
           <t>справочник: Полукомбинезон / брюки зимние</t>
         </is>
       </c>
+      <c r="S13" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T13" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda
+https://www.trakt.ru/</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="13" t="inlineStr"/>
@@ -1250,6 +1371,12 @@
           <t>Спецобъединение «Рефлект-2» 6 112 −10%</t>
         </is>
       </c>
+      <c r="S14" s="16" t="inlineStr">
+        <is>
+          <t>spets.ru</t>
+        </is>
+      </c>
+      <c r="T14" s="13" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="13" t="inlineStr"/>
@@ -1276,7 +1403,7 @@
       <c r="J15" s="15" t="n">
         <v>10550</v>
       </c>
-      <c r="K15" s="16" t="n">
+      <c r="K15" s="17" t="n">
         <v>0.310159487203295</v>
       </c>
       <c r="L15" s="15" t="n">
@@ -1294,6 +1421,12 @@
           <t>Спецобъединение «Рефлект-2» зим. 11 621 −10%</t>
         </is>
       </c>
+      <c r="S15" s="16" t="inlineStr">
+        <is>
+          <t>spets.ru</t>
+        </is>
+      </c>
+      <c r="T15" s="13" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="13" t="inlineStr"/>
@@ -1338,6 +1471,16 @@
           <t>Тракт 11 253 / Спецобъединение 24 199, среднее −10%</t>
         </is>
       </c>
+      <c r="S16" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T16" s="13" t="inlineStr">
+        <is>
+          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="13" t="inlineStr"/>
@@ -1382,6 +1525,16 @@
           <t>Тракт 11 253 / Спецобъединение 24 199, среднее −10%</t>
         </is>
       </c>
+      <c r="S17" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T17" s="13" t="inlineStr">
+        <is>
+          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="13" t="inlineStr"/>
@@ -1426,6 +1579,16 @@
           <t>Тракт 6 731 / Спецобъединение 13 219, среднее −10%</t>
         </is>
       </c>
+      <c r="S18" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T18" s="13" t="inlineStr">
+        <is>
+          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="13" t="inlineStr"/>
@@ -1470,6 +1633,16 @@
           <t>Тракт 6 731 / Спецобъединение 13 219, среднее −10%</t>
         </is>
       </c>
+      <c r="S19" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T19" s="13" t="inlineStr">
+        <is>
+          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="13" t="inlineStr"/>
@@ -1514,6 +1687,16 @@
           <t>Тракт 971 / Фабрикант 1 365</t>
         </is>
       </c>
+      <c r="S20" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T20" s="13" t="inlineStr">
+        <is>
+          <t>https://fabrikant-textile.ru/catalog/spetsodezhda/</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="13" t="inlineStr"/>
@@ -1558,6 +1741,17 @@
           <t>справочник: Футболка</t>
         </is>
       </c>
+      <c r="S21" s="16" t="inlineStr">
+        <is>
+          <t>productcenter.ru</t>
+        </is>
+      </c>
+      <c r="T21" s="13" t="inlineStr">
+        <is>
+          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf
+https://www.trakt.ru/product/12012/</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="13" t="inlineStr"/>
@@ -1602,6 +1796,17 @@
           <t>справочник: Халат рабочий</t>
         </is>
       </c>
+      <c r="S22" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T22" s="13" t="inlineStr">
+        <is>
+          <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/
+https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="13" t="inlineStr"/>
@@ -1646,6 +1851,17 @@
           <t>справочник: Халат рабочий</t>
         </is>
       </c>
+      <c r="S23" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T23" s="13" t="inlineStr">
+        <is>
+          <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/
+https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="13" t="inlineStr"/>
@@ -1688,6 +1904,17 @@
       <c r="R24" s="13" t="inlineStr">
         <is>
           <t>справочник: Халат рабочий</t>
+        </is>
+      </c>
+      <c r="S24" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T24" s="13" t="inlineStr">
+        <is>
+          <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/
+https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
         </is>
       </c>
     </row>
@@ -1750,6 +1977,8 @@
           <t>по позициям ниже</t>
         </is>
       </c>
+      <c r="S25" s="4" t="n"/>
+      <c r="T25" s="4" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="13" t="inlineStr"/>
@@ -1788,6 +2017,17 @@
           <t>справочник: Костюм зимний рабочий (I–III пояс)</t>
         </is>
       </c>
+      <c r="S26" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T26" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda
+https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="13" t="inlineStr"/>
@@ -1826,6 +2066,17 @@
           <t>справочник: Куртка утепленная</t>
         </is>
       </c>
+      <c r="S27" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T27" s="13" t="inlineStr">
+        <is>
+          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
+https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="13" t="inlineStr"/>
@@ -1864,6 +2115,17 @@
           <t>справочник: Полукомбинезон / брюки зимние</t>
         </is>
       </c>
+      <c r="S28" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T28" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda
+https://www.trakt.ru/</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="13" t="inlineStr"/>
@@ -1902,6 +2164,17 @@
           <t>справочник: Куртка утепленная</t>
         </is>
       </c>
+      <c r="S29" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T29" s="13" t="inlineStr">
+        <is>
+          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
+https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="13" t="inlineStr"/>
@@ -1940,6 +2213,17 @@
           <t>справочник: Полукомбинезон / брюки зимние</t>
         </is>
       </c>
+      <c r="S30" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T30" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda
+https://www.trakt.ru/</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="13" t="inlineStr"/>
@@ -1978,6 +2262,17 @@
           <t>справочник: Куртка утепленная</t>
         </is>
       </c>
+      <c r="S31" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T31" s="13" t="inlineStr">
+        <is>
+          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
+https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="13" t="inlineStr"/>
@@ -2002,7 +2297,7 @@
       <c r="J32" s="15" t="n">
         <v>1828.1375</v>
       </c>
-      <c r="K32" s="16" t="n">
+      <c r="K32" s="17" t="n">
         <v>0.3946564569536424</v>
       </c>
       <c r="L32" s="15" t="n"/>
@@ -2016,6 +2311,17 @@
           <t>справочник: Полукомбинезон / брюки зимние</t>
         </is>
       </c>
+      <c r="S32" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T32" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda
+https://www.trakt.ru/</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="13" t="inlineStr"/>
@@ -2054,6 +2360,12 @@
           <t>Тракт, костюм КЩС утепл. 6 215</t>
         </is>
       </c>
+      <c r="S33" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T33" s="13" t="inlineStr"/>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="13" t="inlineStr"/>
@@ -2092,6 +2404,17 @@
           <t>справочник: Костюм сварщика</t>
         </is>
       </c>
+      <c r="S34" s="16" t="inlineStr">
+        <is>
+          <t>ivuniforma.ru</t>
+        </is>
+      </c>
+      <c r="T34" s="13" t="inlineStr">
+        <is>
+          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf
+https://www.trakt.ru/</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="13" t="inlineStr"/>
@@ -2116,7 +2439,7 @@
       <c r="J35" s="15" t="n">
         <v>10550</v>
       </c>
-      <c r="K35" s="17" t="n">
+      <c r="K35" s="18" t="n">
         <v>-0.06490360351266782</v>
       </c>
       <c r="L35" s="15" t="n"/>
@@ -2130,6 +2453,12 @@
           <t>Спецобъединение «Рефлект-2» зим. 11 621 −10%</t>
         </is>
       </c>
+      <c r="S35" s="16" t="inlineStr">
+        <is>
+          <t>spets.ru</t>
+        </is>
+      </c>
+      <c r="T35" s="13" t="inlineStr"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="13" t="inlineStr"/>
@@ -2168,6 +2497,17 @@
           <t>справочник: Жилет утепленный</t>
         </is>
       </c>
+      <c r="S36" s="16" t="inlineStr">
+        <is>
+          <t>ivuniforma.ru</t>
+        </is>
+      </c>
+      <c r="T36" s="13" t="inlineStr">
+        <is>
+          <t>https://www.trakt.ru/product/12021/
+https://www.spets.ru/products/spetsodezhda/odezhda_dlya_okhrannykh_struktur/</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="4" t="n">
@@ -2240,6 +2580,12 @@
           <t>прайс «А-Стандарт» −25 °C 22 800 ₽/т + доставка</t>
         </is>
       </c>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>bicotender.ru</t>
+        </is>
+      </c>
+      <c r="T37" s="8" t="inlineStr"/>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="4" t="n">
@@ -2312,6 +2658,18 @@
           <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410)</t>
         </is>
       </c>
+      <c r="S38" s="7" t="inlineStr">
+        <is>
+          <t>esolk.ru</t>
+        </is>
+      </c>
+      <c r="T38" s="8" t="inlineStr">
+        <is>
+          <t>https://nsmgr.ru/reagenty/tekhnicheskaya-sol/big-begi
+https://sknerud.ru/reagent/sol-texnicheskaya/
+https://vektor-e.ru/sol/</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="4" t="n">
@@ -2365,7 +2723,7 @@
       <c r="M39" s="9" t="n">
         <v>1273942</v>
       </c>
-      <c r="N39" s="16" t="n">
+      <c r="N39" s="17" t="n">
         <v>0.32</v>
       </c>
       <c r="O39" s="12" t="n">
@@ -2382,6 +2740,16 @@
       <c r="R39" s="8" t="inlineStr">
         <is>
           <t>оценка по дилерским прайсам (цен по позициям нет)</t>
+        </is>
+      </c>
+      <c r="S39" s="7" t="inlineStr">
+        <is>
+          <t>specarmatura.ru</t>
+        </is>
+      </c>
+      <c r="T39" s="8" t="inlineStr">
+        <is>
+          <t>https://dn.ru/sharovyi-kran/teplosnabzhenie/flantcevyi-kran/standartnyi/ld/st20/dn100</t>
         </is>
       </c>
     </row>
@@ -2456,6 +2824,12 @@
           <t>оценка по аналогам</t>
         </is>
       </c>
+      <c r="S40" s="8" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T40" s="4" t="n"/>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="4" t="n">
@@ -2508,6 +2882,8 @@
           <t>по позициям ниже</t>
         </is>
       </c>
+      <c r="S41" s="4" t="n"/>
+      <c r="T41" s="4" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="13" t="inlineStr"/>
@@ -2532,7 +2908,7 @@
       <c r="J42" s="15" t="n">
         <v>1144.5</v>
       </c>
-      <c r="K42" s="18" t="n"/>
+      <c r="K42" s="19" t="n"/>
       <c r="L42" s="15" t="n"/>
       <c r="M42" s="15" t="n">
         <v>343350</v>
@@ -2546,6 +2922,12 @@
           <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 3.290 1 091.64 ₽)</t>
         </is>
       </c>
+      <c r="S42" s="16" t="inlineStr">
+        <is>
+          <t>files.technoavia.ru</t>
+        </is>
+      </c>
+      <c r="T42" s="13" t="inlineStr"/>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="13" t="inlineStr"/>
@@ -2570,7 +2952,7 @@
       <c r="J43" s="15" t="n">
         <v>4052.5</v>
       </c>
-      <c r="K43" s="18" t="n"/>
+      <c r="K43" s="19" t="n"/>
       <c r="L43" s="15" t="n"/>
       <c r="M43" s="15" t="n">
         <v>810500</v>
@@ -2582,6 +2964,16 @@
       <c r="R43" s="13" t="inlineStr">
         <is>
           <t>[оценка]: правило клиента 3 500 + антистатическая ткань ~15%</t>
+        </is>
+      </c>
+      <c r="S43" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T43" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
         </is>
       </c>
     </row>
@@ -2608,7 +3000,7 @@
       <c r="J44" s="15" t="n">
         <v>530.5</v>
       </c>
-      <c r="K44" s="18" t="n"/>
+      <c r="K44" s="19" t="n"/>
       <c r="L44" s="15" t="n"/>
       <c r="M44" s="15" t="n">
         <v>106100</v>
@@ -2622,6 +3014,12 @@
           <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 4.025 477.84 ₽)</t>
         </is>
       </c>
+      <c r="S44" s="16" t="inlineStr">
+        <is>
+          <t>files.technoavia.ru</t>
+        </is>
+      </c>
+      <c r="T44" s="13" t="inlineStr"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="13" t="inlineStr"/>
@@ -2646,7 +3044,7 @@
       <c r="J45" s="15" t="n">
         <v>3070.5</v>
       </c>
-      <c r="K45" s="18" t="n"/>
+      <c r="K45" s="19" t="n"/>
       <c r="L45" s="15" t="n"/>
       <c r="M45" s="15" t="n">
         <v>153525</v>
@@ -2660,6 +3058,12 @@
           <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 5.856 «Билд» с мет. носками 3 018.36 ₽)</t>
         </is>
       </c>
+      <c r="S45" s="16" t="inlineStr">
+        <is>
+          <t>files.technoavia.ru</t>
+        </is>
+      </c>
+      <c r="T45" s="13" t="inlineStr"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="4" t="n">
@@ -2712,6 +3116,8 @@
           <t>по позициям ниже</t>
         </is>
       </c>
+      <c r="S46" s="4" t="n"/>
+      <c r="T46" s="4" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="13" t="inlineStr"/>
@@ -2736,7 +3142,7 @@
       <c r="J47" s="15" t="n">
         <v>3552.5</v>
       </c>
-      <c r="K47" s="18" t="n"/>
+      <c r="K47" s="19" t="n"/>
       <c r="L47" s="15" t="n"/>
       <c r="M47" s="15" t="n">
         <v>284200</v>
@@ -2748,6 +3154,16 @@
       <c r="R47" s="13" t="inlineStr">
         <is>
           <t>правило клиента: летний комплект 3 500 ₽</t>
+        </is>
+      </c>
+      <c r="S47" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T47" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
         </is>
       </c>
     </row>
@@ -2774,7 +3190,7 @@
       <c r="J48" s="15" t="n">
         <v>5052.5</v>
       </c>
-      <c r="K48" s="18" t="n"/>
+      <c r="K48" s="19" t="n"/>
       <c r="L48" s="15" t="n"/>
       <c r="M48" s="15" t="n">
         <v>202100</v>
@@ -2786,6 +3202,16 @@
       <c r="R48" s="13" t="inlineStr">
         <is>
           <t>правило клиента: зимний комплект 5 000 ₽</t>
+        </is>
+      </c>
+      <c r="S48" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T48" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
         </is>
       </c>
     </row>
@@ -2812,7 +3238,7 @@
       <c r="J49" s="15" t="n">
         <v>3070.5</v>
       </c>
-      <c r="K49" s="18" t="n"/>
+      <c r="K49" s="19" t="n"/>
       <c r="L49" s="15" t="n"/>
       <c r="M49" s="15" t="n">
         <v>245640</v>
@@ -2826,6 +3252,12 @@
           <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 5.856 «Билд» с мет. носками 3 018.36 ₽)</t>
         </is>
       </c>
+      <c r="S49" s="16" t="inlineStr">
+        <is>
+          <t>files.technoavia.ru</t>
+        </is>
+      </c>
+      <c r="T49" s="13" t="inlineStr"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="13" t="inlineStr"/>
@@ -2850,7 +3282,7 @@
       <c r="J50" s="15" t="n">
         <v>88.5</v>
       </c>
-      <c r="K50" s="18" t="n"/>
+      <c r="K50" s="19" t="n"/>
       <c r="L50" s="15" t="n"/>
       <c r="M50" s="15" t="n">
         <v>132750</v>
@@ -2864,6 +3296,12 @@
           <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 7.002 «Строй» 36 ₽)</t>
         </is>
       </c>
+      <c r="S50" s="16" t="inlineStr">
+        <is>
+          <t>files.technoavia.ru</t>
+        </is>
+      </c>
+      <c r="T50" s="13" t="inlineStr"/>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="13" t="inlineStr"/>
@@ -2888,7 +3326,7 @@
       <c r="J51" s="15" t="n">
         <v>1144.5</v>
       </c>
-      <c r="K51" s="18" t="n"/>
+      <c r="K51" s="19" t="n"/>
       <c r="L51" s="15" t="n"/>
       <c r="M51" s="15" t="n">
         <v>34335</v>
@@ -2902,6 +3340,12 @@
           <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 3.290 1 091.64 ₽)</t>
         </is>
       </c>
+      <c r="S51" s="16" t="inlineStr">
+        <is>
+          <t>files.technoavia.ru</t>
+        </is>
+      </c>
+      <c r="T51" s="13" t="inlineStr"/>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="4" t="n">
@@ -2943,7 +3387,7 @@
       <c r="M52" s="9" t="n">
         <v>561222</v>
       </c>
-      <c r="N52" s="16" t="n">
+      <c r="N52" s="17" t="n">
         <v>0.17</v>
       </c>
       <c r="O52" s="12" t="n">
@@ -2962,6 +3406,8 @@
           <t>по позициям ниже</t>
         </is>
       </c>
+      <c r="S52" s="4" t="n"/>
+      <c r="T52" s="4" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="13" t="inlineStr"/>
@@ -2986,7 +3432,7 @@
       <c r="J53" s="15" t="n">
         <v>12969.86</v>
       </c>
-      <c r="K53" s="16" t="n">
+      <c r="K53" s="17" t="n">
         <v>0.352532265158122</v>
       </c>
       <c r="L53" s="15" t="n"/>
@@ -3000,6 +3446,12 @@
           <t>https://www.trakt.ru/product/142253/</t>
         </is>
       </c>
+      <c r="S53" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T53" s="13" t="inlineStr"/>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="13" t="inlineStr"/>
@@ -3038,6 +3490,12 @@
           <t>https://www.trakt.ru/product/12922/</t>
         </is>
       </c>
+      <c r="S54" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T54" s="13" t="inlineStr"/>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="13" t="inlineStr"/>
@@ -3076,6 +3534,12 @@
           <t>https://www.trakt.ru/product/13076/</t>
         </is>
       </c>
+      <c r="S55" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T55" s="13" t="inlineStr"/>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="13" t="inlineStr"/>
@@ -3100,7 +3564,7 @@
       <c r="J56" s="15" t="n">
         <v>1078.52</v>
       </c>
-      <c r="K56" s="16" t="n">
+      <c r="K56" s="17" t="n">
         <v>0.1989185415165672</v>
       </c>
       <c r="L56" s="15" t="n"/>
@@ -3114,6 +3578,12 @@
           <t>https://www.trakt.ru/product/61070/</t>
         </is>
       </c>
+      <c r="S56" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T56" s="13" t="inlineStr"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="13" t="inlineStr"/>
@@ -3138,7 +3608,7 @@
       <c r="J57" s="15" t="n">
         <v>2047.81</v>
       </c>
-      <c r="K57" s="17" t="n">
+      <c r="K57" s="18" t="n">
         <v>-0.1517491563554556</v>
       </c>
       <c r="L57" s="15" t="n"/>
@@ -3152,6 +3622,12 @@
           <t>https://www.trakt.ru/product/61078/</t>
         </is>
       </c>
+      <c r="S57" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T57" s="13" t="inlineStr"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="13" t="inlineStr"/>
@@ -3190,6 +3666,12 @@
           <t>https://www.trakt.ru/product/61033/</t>
         </is>
       </c>
+      <c r="S58" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T58" s="13" t="inlineStr"/>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="13" t="inlineStr"/>
@@ -3214,7 +3696,7 @@
       <c r="J59" s="15" t="n">
         <v>5030.1</v>
       </c>
-      <c r="K59" s="17" t="n">
+      <c r="K59" s="18" t="n">
         <v>-0.4501523638743381</v>
       </c>
       <c r="L59" s="15" t="n"/>
@@ -3228,6 +3710,12 @@
           <t>https://www.trakt.ru/product/143889/</t>
         </is>
       </c>
+      <c r="S59" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T59" s="13" t="inlineStr"/>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="13" t="inlineStr"/>
@@ -3252,7 +3740,7 @@
       <c r="J60" s="15" t="n">
         <v>33207.83</v>
       </c>
-      <c r="K60" s="16" t="n">
+      <c r="K60" s="17" t="n">
         <v>0.01643353443314751</v>
       </c>
       <c r="L60" s="15" t="n"/>
@@ -3266,6 +3754,12 @@
           <t>https://www.trakt.ru/product/61043/</t>
         </is>
       </c>
+      <c r="S60" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T60" s="13" t="inlineStr"/>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="13" t="inlineStr"/>
@@ -3304,6 +3798,12 @@
           <t>https://www.trakt.ru/product/16450/</t>
         </is>
       </c>
+      <c r="S61" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T61" s="13" t="inlineStr"/>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="4" t="n">
@@ -3345,7 +3845,7 @@
       <c r="M62" s="9" t="n">
         <v>133837274</v>
       </c>
-      <c r="N62" s="16" t="n">
+      <c r="N62" s="17" t="n">
         <v>0.32</v>
       </c>
       <c r="O62" s="12" t="n">
@@ -3364,6 +3864,8 @@
           <t>по позициям ниже</t>
         </is>
       </c>
+      <c r="S62" s="4" t="n"/>
+      <c r="T62" s="4" t="n"/>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="13" t="inlineStr"/>
@@ -3388,7 +3890,7 @@
       <c r="J63" s="15" t="n">
         <v>3552.5</v>
       </c>
-      <c r="K63" s="16" t="n">
+      <c r="K63" s="17" t="n">
         <v>0.2332827584123073</v>
       </c>
       <c r="L63" s="15" t="n"/>
@@ -3402,6 +3904,16 @@
           <t>[правило клиента] летний форменный комплект 3500 ₽</t>
         </is>
       </c>
+      <c r="S63" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T63" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="13" t="inlineStr"/>
@@ -3426,7 +3938,7 @@
       <c r="J64" s="15" t="n">
         <v>5521.15</v>
       </c>
-      <c r="K64" s="17" t="n">
+      <c r="K64" s="18" t="n">
         <v>-0.01310337740883049</v>
       </c>
       <c r="L64" s="15" t="n"/>
@@ -3440,6 +3952,12 @@
           <t>https://www.trakt.ru/product/11930/</t>
         </is>
       </c>
+      <c r="S64" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T64" s="13" t="inlineStr"/>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="13" t="inlineStr"/>
@@ -3478,6 +3996,12 @@
           <t>https://www.trakt.ru/product/138206/</t>
         </is>
       </c>
+      <c r="S65" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T65" s="13" t="inlineStr"/>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="13" t="inlineStr"/>
@@ -3516,6 +4040,12 @@
           <t>https://www.trakt.ru/product/11891/</t>
         </is>
       </c>
+      <c r="S66" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T66" s="13" t="inlineStr"/>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="13" t="inlineStr"/>
@@ -3540,7 +4070,7 @@
       <c r="J67" s="15" t="n">
         <v>3552.5</v>
       </c>
-      <c r="K67" s="16" t="n">
+      <c r="K67" s="17" t="n">
         <v>0.241999116643587</v>
       </c>
       <c r="L67" s="15" t="n"/>
@@ -3554,6 +4084,16 @@
           <t>[правило клиента] летний форменный комплект 3500 ₽</t>
         </is>
       </c>
+      <c r="S67" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T67" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="13" t="inlineStr"/>
@@ -3578,7 +4118,7 @@
       <c r="J68" s="15" t="n">
         <v>1480.51</v>
       </c>
-      <c r="K68" s="17" t="n">
+      <c r="K68" s="18" t="n">
         <v>-0.1650036983994587</v>
       </c>
       <c r="L68" s="15" t="n"/>
@@ -3592,6 +4132,12 @@
           <t>https://www.trakt.ru/product/135628/</t>
         </is>
       </c>
+      <c r="S68" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T68" s="13" t="inlineStr"/>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="13" t="inlineStr"/>
@@ -3630,6 +4176,12 @@
           <t>[оценка] костюм антипорезный летний 7–11 тыс. ₽</t>
         </is>
       </c>
+      <c r="S69" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T69" s="14" t="n"/>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="13" t="inlineStr"/>
@@ -3654,7 +4206,7 @@
       <c r="J70" s="15" t="n">
         <v>5937.17</v>
       </c>
-      <c r="K70" s="16" t="n">
+      <c r="K70" s="17" t="n">
         <v>0.3096137343048311</v>
       </c>
       <c r="L70" s="15" t="n"/>
@@ -3668,6 +4220,12 @@
           <t>https://www.trakt.ru/product/16725/</t>
         </is>
       </c>
+      <c r="S70" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T70" s="13" t="inlineStr"/>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="13" t="inlineStr"/>
@@ -3706,6 +4264,12 @@
           <t>https://www.trakt.ru/product/11992/</t>
         </is>
       </c>
+      <c r="S71" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T71" s="13" t="inlineStr"/>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="13" t="inlineStr"/>
@@ -3744,6 +4308,12 @@
           <t>https://www.trakt.ru/product/11891/</t>
         </is>
       </c>
+      <c r="S72" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T72" s="13" t="inlineStr"/>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="13" t="inlineStr"/>
@@ -3768,7 +4338,7 @@
       <c r="J73" s="15" t="n">
         <v>12912.52</v>
       </c>
-      <c r="K73" s="17" t="n">
+      <c r="K73" s="18" t="n">
         <v>-0.08509665643687174</v>
       </c>
       <c r="L73" s="15" t="n"/>
@@ -3782,6 +4352,12 @@
           <t>https://www.trakt.ru/product/12592/</t>
         </is>
       </c>
+      <c r="S73" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T73" s="13" t="inlineStr"/>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="13" t="inlineStr"/>
@@ -3806,7 +4382,7 @@
       <c r="J74" s="15" t="n">
         <v>84.83</v>
       </c>
-      <c r="K74" s="17" t="n">
+      <c r="K74" s="18" t="n">
         <v>-0.5107747105966162</v>
       </c>
       <c r="L74" s="15" t="n"/>
@@ -3820,6 +4396,12 @@
           <t>https://www.trakt.ru/product/13074/</t>
         </is>
       </c>
+      <c r="S74" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T74" s="13" t="inlineStr"/>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="13" t="inlineStr"/>
@@ -3858,6 +4440,12 @@
           <t>https://www.trakt.ru/product/16651/</t>
         </is>
       </c>
+      <c r="S75" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T75" s="13" t="inlineStr"/>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="13" t="inlineStr"/>
@@ -3882,7 +4470,7 @@
       <c r="J76" s="15" t="n">
         <v>5052.5</v>
       </c>
-      <c r="K76" s="16" t="n">
+      <c r="K76" s="17" t="n">
         <v>0.3670227959489459</v>
       </c>
       <c r="L76" s="15" t="n"/>
@@ -3896,6 +4484,16 @@
           <t>[правило клиента] зимний форменный комплект 5000 ₽</t>
         </is>
       </c>
+      <c r="S76" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T76" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="13" t="inlineStr"/>
@@ -3920,7 +4518,7 @@
       <c r="J77" s="15" t="n">
         <v>5052.5</v>
       </c>
-      <c r="K77" s="16" t="n">
+      <c r="K77" s="17" t="n">
         <v>0.383904575628838</v>
       </c>
       <c r="L77" s="15" t="n"/>
@@ -3934,6 +4532,16 @@
           <t>[правило клиента] зимний форменный комплект 5000 ₽</t>
         </is>
       </c>
+      <c r="S77" s="16" t="inlineStr">
+        <is>
+          <t>fabrikant-textile.ru</t>
+        </is>
+      </c>
+      <c r="T77" s="13" t="inlineStr">
+        <is>
+          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="13" t="inlineStr"/>
@@ -3972,6 +4580,12 @@
           <t>https://www.trakt.ru/product/12027/</t>
         </is>
       </c>
+      <c r="S78" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T78" s="13" t="inlineStr"/>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="13" t="inlineStr"/>
@@ -3996,7 +4610,7 @@
       <c r="J79" s="15" t="n">
         <v>1753.18</v>
       </c>
-      <c r="K79" s="17" t="n">
+      <c r="K79" s="18" t="n">
         <v>-0.2528620635442424</v>
       </c>
       <c r="L79" s="15" t="n"/>
@@ -4010,6 +4624,12 @@
           <t>https://www.trakt.ru/product/12520/</t>
         </is>
       </c>
+      <c r="S79" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T79" s="13" t="inlineStr"/>
     </row>
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="13" t="inlineStr"/>
@@ -4048,6 +4668,12 @@
           <t>[оценка] костюм антипорезный утепл. (бензопильщика) 9–14 тыс. ₽ (energocontract.ru/catalog/chain-saw — цены по запросу)</t>
         </is>
       </c>
+      <c r="S80" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T80" s="14" t="n"/>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="13" t="inlineStr"/>
@@ -4086,6 +4712,12 @@
           <t>https://www.trakt.ru/product/11812/</t>
         </is>
       </c>
+      <c r="S81" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T81" s="13" t="inlineStr"/>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="13" t="inlineStr"/>
@@ -4110,7 +4742,7 @@
       <c r="J82" s="15" t="n">
         <v>1013.25</v>
       </c>
-      <c r="K82" s="16" t="n">
+      <c r="K82" s="17" t="n">
         <v>0.1551039807881527</v>
       </c>
       <c r="L82" s="15" t="n"/>
@@ -4124,6 +4756,12 @@
           <t>https://www.trakt.ru/catalog/zashhita-ruk/kozhanye-perchatki/ (краги РУССКИЕ ЛЬВЫ утепл.)</t>
         </is>
       </c>
+      <c r="S82" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T82" s="13" t="inlineStr"/>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="13" t="inlineStr"/>
@@ -4162,6 +4800,12 @@
           <t>[оценка] перчатки бензопильщика 1.8–3 тыс. ₽</t>
         </is>
       </c>
+      <c r="S83" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T83" s="14" t="n"/>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="13" t="inlineStr"/>
@@ -4186,7 +4830,7 @@
       <c r="J84" s="15" t="n">
         <v>856.48</v>
       </c>
-      <c r="K84" s="17" t="n">
+      <c r="K84" s="18" t="n">
         <v>-0.2165909090909091</v>
       </c>
       <c r="L84" s="15" t="n"/>
@@ -4200,6 +4844,12 @@
           <t>https://www.trakt.ru/product/12001/</t>
         </is>
       </c>
+      <c r="S84" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T84" s="13" t="inlineStr"/>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="13" t="inlineStr"/>
@@ -4238,6 +4888,12 @@
           <t>https://www.trakt.ru/product/12913/</t>
         </is>
       </c>
+      <c r="S85" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T85" s="13" t="inlineStr"/>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="13" t="inlineStr"/>
@@ -4276,6 +4932,12 @@
           <t>[оценка] перчатки бензопильщика утепл. 2–3.5 тыс. ₽</t>
         </is>
       </c>
+      <c r="S86" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T86" s="14" t="n"/>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="13" t="inlineStr"/>
@@ -4314,6 +4976,12 @@
           <t>[оценка] перчатки резиновые технические 80–150 ₽</t>
         </is>
       </c>
+      <c r="S87" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T87" s="14" t="n"/>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="13" t="inlineStr"/>
@@ -4352,6 +5020,12 @@
           <t>[оценка] нарукавники х/б/ПВХ 100–200 ₽</t>
         </is>
       </c>
+      <c r="S88" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T88" s="14" t="n"/>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="13" t="inlineStr"/>
@@ -4376,7 +5050,7 @@
       <c r="J89" s="15" t="n">
         <v>311.14</v>
       </c>
-      <c r="K89" s="16" t="n">
+      <c r="K89" s="17" t="n">
         <v>0.1450788591526076</v>
       </c>
       <c r="L89" s="15" t="n"/>
@@ -4390,6 +5064,12 @@
           <t>https://www.trakt.ru/product/11708/</t>
         </is>
       </c>
+      <c r="S89" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T89" s="13" t="inlineStr"/>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="13" t="inlineStr"/>
@@ -4414,7 +5094,7 @@
       <c r="J90" s="15" t="n">
         <v>366.04</v>
       </c>
-      <c r="K90" s="16" t="n">
+      <c r="K90" s="17" t="n">
         <v>0.3309449826357156</v>
       </c>
       <c r="L90" s="15" t="n"/>
@@ -4428,6 +5108,12 @@
           <t>https://www.trakt.ru/product/11707/</t>
         </is>
       </c>
+      <c r="S90" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T90" s="13" t="inlineStr"/>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="13" t="inlineStr"/>
@@ -4466,6 +5152,12 @@
           <t>[оценка] накомарник х/б 150–300 ₽</t>
         </is>
       </c>
+      <c r="S91" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T91" s="14" t="n"/>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="13" t="inlineStr"/>
@@ -4490,7 +5182,7 @@
       <c r="J92" s="15" t="n">
         <v>317.85</v>
       </c>
-      <c r="K92" s="16" t="n">
+      <c r="K92" s="17" t="n">
         <v>0.2126579142927916</v>
       </c>
       <c r="L92" s="15" t="n"/>
@@ -4504,6 +5196,12 @@
           <t>https://www.trakt.ru/product/13005/</t>
         </is>
       </c>
+      <c r="S92" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T92" s="13" t="inlineStr"/>
     </row>
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="13" t="inlineStr"/>
@@ -4528,7 +5226,7 @@
       <c r="J93" s="15" t="n">
         <v>1028.5</v>
       </c>
-      <c r="K93" s="16" t="n">
+      <c r="K93" s="17" t="n">
         <v>0.2467905294070261</v>
       </c>
       <c r="L93" s="15" t="n"/>
@@ -4542,6 +5240,12 @@
           <t>https://www.trakt.ru/product/61033/</t>
         </is>
       </c>
+      <c r="S93" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T93" s="13" t="inlineStr"/>
     </row>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="13" t="inlineStr"/>
@@ -4580,6 +5284,12 @@
           <t>[оценка] наплечники брезентовые 200–400 ₽</t>
         </is>
       </c>
+      <c r="S94" s="13" t="inlineStr">
+        <is>
+          <t>нет открытой цены — оценка</t>
+        </is>
+      </c>
+      <c r="T94" s="14" t="n"/>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="13" t="inlineStr"/>
@@ -4618,6 +5328,12 @@
           <t>https://www.trakt.ru/product/11961/</t>
         </is>
       </c>
+      <c r="S95" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T95" s="13" t="inlineStr"/>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="13" t="inlineStr"/>
@@ -4642,7 +5358,7 @@
       <c r="J96" s="15" t="n">
         <v>1028.5</v>
       </c>
-      <c r="K96" s="16" t="n">
+      <c r="K96" s="17" t="n">
         <v>0.3454047861507129</v>
       </c>
       <c r="L96" s="15" t="n"/>
@@ -4656,6 +5372,12 @@
           <t>https://www.trakt.ru/product/61033/</t>
         </is>
       </c>
+      <c r="S96" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T96" s="13" t="inlineStr"/>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="13" t="inlineStr"/>
@@ -4680,7 +5402,7 @@
       <c r="J97" s="15" t="n">
         <v>1786.12</v>
       </c>
-      <c r="K97" s="16" t="n">
+      <c r="K97" s="17" t="n">
         <v>0.1493127327802174</v>
       </c>
       <c r="L97" s="15" t="n"/>
@@ -4694,6 +5416,12 @@
           <t>https://www.trakt.ru/product/12190/</t>
         </is>
       </c>
+      <c r="S97" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T97" s="13" t="inlineStr"/>
     </row>
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="13" t="inlineStr"/>
@@ -4718,7 +5446,7 @@
       <c r="J98" s="15" t="n">
         <v>2477.86</v>
       </c>
-      <c r="K98" s="16" t="n">
+      <c r="K98" s="17" t="n">
         <v>0.3180533423604173</v>
       </c>
       <c r="L98" s="15" t="n"/>
@@ -4732,6 +5460,12 @@
           <t>https://www.trakt.ru/product/13076/</t>
         </is>
       </c>
+      <c r="S98" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T98" s="13" t="inlineStr"/>
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="13" t="inlineStr"/>
@@ -4756,7 +5490,7 @@
       <c r="J99" s="15" t="n">
         <v>3541.7</v>
       </c>
-      <c r="K99" s="16" t="n">
+      <c r="K99" s="17" t="n">
         <v>0.2083516807746383</v>
       </c>
       <c r="L99" s="15" t="n"/>
@@ -4770,6 +5504,12 @@
           <t>https://www.trakt.ru/product/61013/</t>
         </is>
       </c>
+      <c r="S99" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T99" s="13" t="inlineStr"/>
     </row>
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="13" t="inlineStr"/>
@@ -4794,7 +5534,7 @@
       <c r="J100" s="15" t="n">
         <v>4516.48</v>
       </c>
-      <c r="K100" s="17" t="n">
+      <c r="K100" s="18" t="n">
         <v>-0.1232985054952706</v>
       </c>
       <c r="L100" s="15" t="n"/>
@@ -4808,6 +5548,12 @@
           <t>https://www.trakt.ru/product/16450/</t>
         </is>
       </c>
+      <c r="S100" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T100" s="13" t="inlineStr"/>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="13" t="inlineStr"/>
@@ -4832,7 +5578,7 @@
       <c r="J101" s="15" t="n">
         <v>1961.19</v>
       </c>
-      <c r="K101" s="16" t="n">
+      <c r="K101" s="17" t="n">
         <v>0.387128125</v>
       </c>
       <c r="L101" s="15" t="n"/>
@@ -4846,6 +5592,12 @@
           <t>https://www.trakt.ru/product/12193/</t>
         </is>
       </c>
+      <c r="S101" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T101" s="13" t="inlineStr"/>
     </row>
     <row r="102" ht="30" customHeight="1">
       <c r="A102" s="13" t="inlineStr"/>
@@ -4884,6 +5636,12 @@
           <t>https://www.trakt.ru/product/16585/</t>
         </is>
       </c>
+      <c r="S102" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T102" s="13" t="inlineStr"/>
     </row>
     <row r="103" ht="30" customHeight="1">
       <c r="A103" s="13" t="inlineStr"/>
@@ -4908,7 +5666,7 @@
       <c r="J103" s="15" t="n">
         <v>4545.15</v>
       </c>
-      <c r="K103" s="16" t="n">
+      <c r="K103" s="17" t="n">
         <v>0.2504502097680678</v>
       </c>
       <c r="L103" s="15" t="n"/>
@@ -4922,6 +5680,12 @@
           <t>https://www.trakt.ru/product/13084/</t>
         </is>
       </c>
+      <c r="S103" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T103" s="13" t="inlineStr"/>
     </row>
     <row r="104" ht="30" customHeight="1">
       <c r="A104" s="13" t="inlineStr"/>
@@ -4946,7 +5710,7 @@
       <c r="J104" s="15" t="n">
         <v>2156.1</v>
       </c>
-      <c r="K104" s="16" t="n">
+      <c r="K104" s="17" t="n">
         <v>0.2340021884636702</v>
       </c>
       <c r="L104" s="15" t="n"/>
@@ -4960,51 +5724,145 @@
           <t>https://www.trakt.ru/catalog/specobuv/valenki/12196/</t>
         </is>
       </c>
+      <c r="S104" s="16" t="inlineStr">
+        <is>
+          <t>trakt.ru</t>
+        </is>
+      </c>
+      <c r="T104" s="13" t="inlineStr"/>
     </row>
     <row r="105" ht="30" customHeight="1">
-      <c r="A105" s="19" t="inlineStr"/>
-      <c r="B105" s="19" t="inlineStr">
+      <c r="A105" s="20" t="inlineStr"/>
+      <c r="B105" s="20" t="inlineStr">
         <is>
           <t>ИТОГО — обычные условия</t>
         </is>
       </c>
-      <c r="C105" s="19" t="inlineStr"/>
-      <c r="D105" s="19" t="inlineStr"/>
-      <c r="E105" s="19" t="inlineStr"/>
-      <c r="F105" s="19" t="inlineStr"/>
-      <c r="G105" s="19" t="inlineStr"/>
-      <c r="H105" s="19" t="inlineStr"/>
-      <c r="I105" s="19" t="inlineStr"/>
-      <c r="J105" s="19" t="inlineStr"/>
-      <c r="K105" s="19" t="inlineStr"/>
-      <c r="L105" s="20" t="n">
+      <c r="C105" s="20" t="inlineStr"/>
+      <c r="D105" s="20" t="inlineStr"/>
+      <c r="E105" s="20" t="inlineStr"/>
+      <c r="F105" s="20" t="inlineStr"/>
+      <c r="G105" s="20" t="inlineStr"/>
+      <c r="H105" s="20" t="inlineStr"/>
+      <c r="I105" s="20" t="inlineStr"/>
+      <c r="J105" s="20" t="inlineStr"/>
+      <c r="K105" s="20" t="inlineStr"/>
+      <c r="L105" s="21" t="n">
         <v>22113376</v>
       </c>
-      <c r="M105" s="20" t="n">
+      <c r="M105" s="21" t="n">
         <v>9437915</v>
       </c>
-      <c r="N105" s="21" t="n"/>
-      <c r="O105" s="20" t="n">
+      <c r="N105" s="22" t="n"/>
+      <c r="O105" s="21" t="n">
         <v>8097652</v>
       </c>
-      <c r="P105" s="21" t="n"/>
-      <c r="Q105" s="21" t="n"/>
-      <c r="R105" s="21" t="n"/>
+      <c r="P105" s="22" t="n"/>
+      <c r="Q105" s="22" t="n"/>
+      <c r="R105" s="22" t="n"/>
+      <c r="S105" s="22" t="n"/>
+      <c r="T105" s="22" t="n"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S37" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S39" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S42" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S43" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S44" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S45" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S47" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S48" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S50" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S51" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S53" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S54" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S55" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S56" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S57" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S58" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S59" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S60" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S61" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S63" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S64" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S65" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S66" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S67" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S68" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S70" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S71" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S72" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S73" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S74" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S75" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S76" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S77" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S78" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S79" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S81" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S82" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S89" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S90" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S92" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S93" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S95" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S96" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S97" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S98" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S99" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S100" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S101" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S102" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S103" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S104" r:id="rId98"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Itog: compact extra source domains
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/ITOG_LOTS_1410.xlsx
+++ b/ITOG_LOTS_1410.xlsx
@@ -792,9 +792,7 @@
       </c>
       <c r="T4" s="8" t="inlineStr">
         <is>
-          <t>https://nsmgr.ru/reagenty/tekhnicheskaya-sol/big-begi
-https://sknerud.ru/reagent/sol-texnicheskaya/
-https://vektor-e.ru/sol/</t>
+          <t>nsmgr.ru, sknerud.ru, vektor-e.ru</t>
         </is>
       </c>
     </row>
@@ -876,9 +874,7 @@
       </c>
       <c r="T5" s="8" t="inlineStr">
         <is>
-          <t>https://nsmgr.ru/reagenty/tekhnicheskaya-sol/big-begi
-https://sknerud.ru/reagent/sol-texnicheskaya/
-https://vektor-e.ru/sol/</t>
+          <t>nsmgr.ru, sknerud.ru, vektor-e.ru</t>
         </is>
       </c>
     </row>
@@ -994,8 +990,7 @@
       </c>
       <c r="T7" s="13" t="inlineStr">
         <is>
-          <t>https://www.trakt.ru/product/138206/
-https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+          <t>trakt.ru, spets.ru</t>
         </is>
       </c>
     </row>
@@ -1049,8 +1044,7 @@
       </c>
       <c r="T8" s="13" t="inlineStr">
         <is>
-          <t>https://www.trakt.ru/product/12021/
-https://www.spets.ru/products/spetsodezhda/odezhda_dlya_okhrannykh_struktur/</t>
+          <t>trakt.ru, spets.ru</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1098,7 @@
       </c>
       <c r="T9" s="13" t="inlineStr">
         <is>
-          <t>https://ivsoteks.ru/specodejda</t>
+          <t>ivsoteks.ru</t>
         </is>
       </c>
     </row>
@@ -1158,8 +1152,7 @@
       </c>
       <c r="T10" s="13" t="inlineStr">
         <is>
-          <t>https://ivsoteks.ru/specodejda
-https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+          <t>ivsoteks.ru, files.technoavia.ru</t>
         </is>
       </c>
     </row>
@@ -1213,8 +1206,7 @@
       </c>
       <c r="T11" s="13" t="inlineStr">
         <is>
-          <t>https://ivsoteks.ru/specodejda
-https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+          <t>ivsoteks.ru, files.technoavia.ru</t>
         </is>
       </c>
     </row>
@@ -1268,8 +1260,7 @@
       </c>
       <c r="T12" s="13" t="inlineStr">
         <is>
-          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
-https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+          <t>specteks37.ru, ivuniforma.ru</t>
         </is>
       </c>
     </row>
@@ -1323,8 +1314,7 @@
       </c>
       <c r="T13" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda
-https://www.trakt.ru/</t>
+          <t>spec-standart.ru, trakt.ru</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1468,7 @@
       </c>
       <c r="T16" s="13" t="inlineStr">
         <is>
-          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+          <t>spets.ru</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1522,7 @@
       </c>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+          <t>spets.ru</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1576,7 @@
       </c>
       <c r="T18" s="13" t="inlineStr">
         <is>
-          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+          <t>spets.ru</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1630,7 @@
       </c>
       <c r="T19" s="13" t="inlineStr">
         <is>
-          <t>https://www.spets.ru/products/spetsodezhda/odezhda_spetsialnaya/</t>
+          <t>spets.ru</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1684,7 @@
       </c>
       <c r="T20" s="13" t="inlineStr">
         <is>
-          <t>https://fabrikant-textile.ru/catalog/spetsodezhda/</t>
+          <t>fabrikant-textile.ru</t>
         </is>
       </c>
     </row>
@@ -1748,8 +1738,7 @@
       </c>
       <c r="T21" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf
-https://www.trakt.ru/product/12012/</t>
+          <t>files.technoavia.ru, trakt.ru</t>
         </is>
       </c>
     </row>
@@ -1803,8 +1792,7 @@
       </c>
       <c r="T22" s="13" t="inlineStr">
         <is>
-          <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/
-https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+          <t>ivuniforma.ru, files.technoavia.ru</t>
         </is>
       </c>
     </row>
@@ -1858,8 +1846,7 @@
       </c>
       <c r="T23" s="13" t="inlineStr">
         <is>
-          <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/
-https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+          <t>ivuniforma.ru, files.technoavia.ru</t>
         </is>
       </c>
     </row>
@@ -1913,8 +1900,7 @@
       </c>
       <c r="T24" s="13" t="inlineStr">
         <is>
-          <t>https://www.ivuniforma.ru/catalog/rabochaya-odezhda/letnyaya-spetsodezhda/khalati/
-https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf</t>
+          <t>ivuniforma.ru, files.technoavia.ru</t>
         </is>
       </c>
     </row>
@@ -2024,8 +2010,7 @@
       </c>
       <c r="T26" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda
-https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/</t>
+          <t>spec-standart.ru, specteks37.ru</t>
         </is>
       </c>
     </row>
@@ -2073,8 +2058,7 @@
       </c>
       <c r="T27" s="13" t="inlineStr">
         <is>
-          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
-https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+          <t>specteks37.ru, ivuniforma.ru</t>
         </is>
       </c>
     </row>
@@ -2122,8 +2106,7 @@
       </c>
       <c r="T28" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda
-https://www.trakt.ru/</t>
+          <t>spec-standart.ru, trakt.ru</t>
         </is>
       </c>
     </row>
@@ -2171,8 +2154,7 @@
       </c>
       <c r="T29" s="13" t="inlineStr">
         <is>
-          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
-https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+          <t>specteks37.ru, ivuniforma.ru</t>
         </is>
       </c>
     </row>
@@ -2220,8 +2202,7 @@
       </c>
       <c r="T30" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda
-https://www.trakt.ru/</t>
+          <t>spec-standart.ru, trakt.ru</t>
         </is>
       </c>
     </row>
@@ -2269,8 +2250,7 @@
       </c>
       <c r="T31" s="13" t="inlineStr">
         <is>
-          <t>https://www.specteks37.ru/katalog/zimnyaya-spetsodezhda/
-https://www.ivuniforma.ru/catalog/rabochaya-odezhda/zimnjaja/</t>
+          <t>specteks37.ru, ivuniforma.ru</t>
         </is>
       </c>
     </row>
@@ -2318,8 +2298,7 @@
       </c>
       <c r="T32" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda
-https://www.trakt.ru/</t>
+          <t>spec-standart.ru, trakt.ru</t>
         </is>
       </c>
     </row>
@@ -2411,8 +2390,7 @@
       </c>
       <c r="T34" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf
-https://www.trakt.ru/</t>
+          <t>files.technoavia.ru, trakt.ru</t>
         </is>
       </c>
     </row>
@@ -2504,8 +2482,7 @@
       </c>
       <c r="T36" s="13" t="inlineStr">
         <is>
-          <t>https://www.trakt.ru/product/12021/
-https://www.spets.ru/products/spetsodezhda/odezhda_dlya_okhrannykh_struktur/</t>
+          <t>trakt.ru, spets.ru</t>
         </is>
       </c>
     </row>
@@ -2665,9 +2642,7 @@
       </c>
       <c r="T38" s="8" t="inlineStr">
         <is>
-          <t>https://nsmgr.ru/reagenty/tekhnicheskaya-sol/big-begi
-https://sknerud.ru/reagent/sol-texnicheskaya/
-https://vektor-e.ru/sol/</t>
+          <t>nsmgr.ru, sknerud.ru, vektor-e.ru</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2724,7 @@
       </c>
       <c r="T39" s="8" t="inlineStr">
         <is>
-          <t>https://dn.ru/sharovyi-kran/teplosnabzhenie/flantcevyi-kran/standartnyi/ld/st20/dn100</t>
+          <t>dn.ru</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2948,7 @@
       </c>
       <c r="T43" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>
@@ -3163,7 +3138,7 @@
       </c>
       <c r="T47" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3186,7 @@
       </c>
       <c r="T48" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3886,7 @@
       </c>
       <c r="T63" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4066,7 @@
       </c>
       <c r="T67" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4466,7 @@
       </c>
       <c r="T76" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>
@@ -4539,7 +4514,7 @@
       </c>
       <c r="T77" s="13" t="inlineStr">
         <is>
-          <t>https://spec-standart.ru/zimnyaya-specodezhda</t>
+          <t>spec-standart.ru</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Itog: trim source text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/ITOG_LOTS_1410.xlsx
+++ b/ITOG_LOTS_1410.xlsx
@@ -782,7 +782,7 @@
       </c>
       <c r="R4" s="8" t="inlineStr">
         <is>
-          <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410)</t>
+          <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410</t>
         </is>
       </c>
       <c r="S4" s="7" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="R5" s="8" t="inlineStr">
         <is>
-          <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410)</t>
+          <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410</t>
         </is>
       </c>
       <c r="S5" s="7" t="inlineStr">
@@ -2000,7 +2000,7 @@
       <c r="Q26" s="13" t="inlineStr"/>
       <c r="R26" s="13" t="inlineStr">
         <is>
-          <t>справочник: Костюм зимний рабочий (I–III пояс)</t>
+          <t>справочник: Костюм зимний рабочий (I–III пояс</t>
         </is>
       </c>
       <c r="S26" s="16" t="inlineStr">
@@ -2632,7 +2632,7 @@
       </c>
       <c r="R38" s="8" t="inlineStr">
         <is>
-          <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410)</t>
+          <t>средняя рыночная с доставкой: завод вагоном / склад авто (SALT_STRATEGY_1410</t>
         </is>
       </c>
       <c r="S38" s="7" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="R39" s="8" t="inlineStr">
         <is>
-          <t>оценка по дилерским прайсам (цен по позициям нет)</t>
+          <t>оценка по дилерским прайсам (цен по позициям нет</t>
         </is>
       </c>
       <c r="S39" s="7" t="inlineStr">
@@ -2894,7 +2894,7 @@
       <c r="Q42" s="13" t="inlineStr"/>
       <c r="R42" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 3.290 1 091.64 ₽)</t>
+          <t>арт. 3.290 1 091.64 ₽</t>
         </is>
       </c>
       <c r="S42" s="16" t="inlineStr">
@@ -2986,7 +2986,7 @@
       <c r="Q44" s="13" t="inlineStr"/>
       <c r="R44" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 4.025 477.84 ₽)</t>
+          <t>арт. 4.025 477.84 ₽</t>
         </is>
       </c>
       <c r="S44" s="16" t="inlineStr">
@@ -3030,7 +3030,7 @@
       <c r="Q45" s="13" t="inlineStr"/>
       <c r="R45" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 5.856 «Билд» с мет. носками 3 018.36 ₽)</t>
+          <t>арт. 5.856 «Билд» с мет. носками 3 018.36 ₽</t>
         </is>
       </c>
       <c r="S45" s="16" t="inlineStr">
@@ -3224,7 +3224,7 @@
       <c r="Q49" s="13" t="inlineStr"/>
       <c r="R49" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 5.856 «Билд» с мет. носками 3 018.36 ₽)</t>
+          <t>арт. 5.856 «Билд» с мет. носками 3 018.36 ₽</t>
         </is>
       </c>
       <c r="S49" s="16" t="inlineStr">
@@ -3268,7 +3268,7 @@
       <c r="Q50" s="13" t="inlineStr"/>
       <c r="R50" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 7.002 «Строй» 36 ₽)</t>
+          <t>арт. 7.002 «Строй» 36 ₽</t>
         </is>
       </c>
       <c r="S50" s="16" t="inlineStr">
@@ -3312,7 +3312,7 @@
       <c r="Q51" s="13" t="inlineStr"/>
       <c r="R51" s="13" t="inlineStr">
         <is>
-          <t>https://files.technoavia.ru/files/price/11/price_Technoavia_moscow_2025_06_27_08_46_34.pdf (арт. 3.290 1 091.64 ₽)</t>
+          <t>арт. 3.290 1 091.64 ₽</t>
         </is>
       </c>
       <c r="S51" s="16" t="inlineStr">
@@ -3416,11 +3416,7 @@
       <c r="O53" s="14" t="n"/>
       <c r="P53" s="14" t="n"/>
       <c r="Q53" s="13" t="inlineStr"/>
-      <c r="R53" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/142253/</t>
-        </is>
-      </c>
+      <c r="R53" s="13" t="inlineStr"/>
       <c r="S53" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3460,11 +3456,7 @@
       <c r="O54" s="14" t="n"/>
       <c r="P54" s="14" t="n"/>
       <c r="Q54" s="13" t="inlineStr"/>
-      <c r="R54" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12922/</t>
-        </is>
-      </c>
+      <c r="R54" s="13" t="inlineStr"/>
       <c r="S54" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3504,11 +3496,7 @@
       <c r="O55" s="14" t="n"/>
       <c r="P55" s="14" t="n"/>
       <c r="Q55" s="13" t="inlineStr"/>
-      <c r="R55" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/13076/</t>
-        </is>
-      </c>
+      <c r="R55" s="13" t="inlineStr"/>
       <c r="S55" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3548,11 +3536,7 @@
       <c r="O56" s="14" t="n"/>
       <c r="P56" s="14" t="n"/>
       <c r="Q56" s="13" t="inlineStr"/>
-      <c r="R56" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61070/</t>
-        </is>
-      </c>
+      <c r="R56" s="13" t="inlineStr"/>
       <c r="S56" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3592,11 +3576,7 @@
       <c r="O57" s="14" t="n"/>
       <c r="P57" s="14" t="n"/>
       <c r="Q57" s="13" t="inlineStr"/>
-      <c r="R57" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61078/</t>
-        </is>
-      </c>
+      <c r="R57" s="13" t="inlineStr"/>
       <c r="S57" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3636,11 +3616,7 @@
       <c r="O58" s="14" t="n"/>
       <c r="P58" s="14" t="n"/>
       <c r="Q58" s="13" t="inlineStr"/>
-      <c r="R58" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61033/</t>
-        </is>
-      </c>
+      <c r="R58" s="13" t="inlineStr"/>
       <c r="S58" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3680,11 +3656,7 @@
       <c r="O59" s="14" t="n"/>
       <c r="P59" s="14" t="n"/>
       <c r="Q59" s="13" t="inlineStr"/>
-      <c r="R59" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/143889/</t>
-        </is>
-      </c>
+      <c r="R59" s="13" t="inlineStr"/>
       <c r="S59" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3724,11 +3696,7 @@
       <c r="O60" s="14" t="n"/>
       <c r="P60" s="14" t="n"/>
       <c r="Q60" s="13" t="inlineStr"/>
-      <c r="R60" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61043/</t>
-        </is>
-      </c>
+      <c r="R60" s="13" t="inlineStr"/>
       <c r="S60" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3768,11 +3736,7 @@
       <c r="O61" s="14" t="n"/>
       <c r="P61" s="14" t="n"/>
       <c r="Q61" s="13" t="inlineStr"/>
-      <c r="R61" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/16450/</t>
-        </is>
-      </c>
+      <c r="R61" s="13" t="inlineStr"/>
       <c r="S61" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3922,11 +3886,7 @@
       <c r="O64" s="14" t="n"/>
       <c r="P64" s="14" t="n"/>
       <c r="Q64" s="13" t="inlineStr"/>
-      <c r="R64" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11930/</t>
-        </is>
-      </c>
+      <c r="R64" s="13" t="inlineStr"/>
       <c r="S64" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -3966,11 +3926,7 @@
       <c r="O65" s="14" t="n"/>
       <c r="P65" s="14" t="n"/>
       <c r="Q65" s="13" t="inlineStr"/>
-      <c r="R65" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/138206/</t>
-        </is>
-      </c>
+      <c r="R65" s="13" t="inlineStr"/>
       <c r="S65" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4010,11 +3966,7 @@
       <c r="O66" s="14" t="n"/>
       <c r="P66" s="14" t="n"/>
       <c r="Q66" s="13" t="inlineStr"/>
-      <c r="R66" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11891/</t>
-        </is>
-      </c>
+      <c r="R66" s="13" t="inlineStr"/>
       <c r="S66" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4102,11 +4054,7 @@
       <c r="O68" s="14" t="n"/>
       <c r="P68" s="14" t="n"/>
       <c r="Q68" s="13" t="inlineStr"/>
-      <c r="R68" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/135628/</t>
-        </is>
-      </c>
+      <c r="R68" s="13" t="inlineStr"/>
       <c r="S68" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4190,11 +4138,7 @@
       <c r="O70" s="14" t="n"/>
       <c r="P70" s="14" t="n"/>
       <c r="Q70" s="13" t="inlineStr"/>
-      <c r="R70" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/16725/</t>
-        </is>
-      </c>
+      <c r="R70" s="13" t="inlineStr"/>
       <c r="S70" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4234,11 +4178,7 @@
       <c r="O71" s="14" t="n"/>
       <c r="P71" s="14" t="n"/>
       <c r="Q71" s="13" t="inlineStr"/>
-      <c r="R71" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11992/</t>
-        </is>
-      </c>
+      <c r="R71" s="13" t="inlineStr"/>
       <c r="S71" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4278,11 +4218,7 @@
       <c r="O72" s="14" t="n"/>
       <c r="P72" s="14" t="n"/>
       <c r="Q72" s="13" t="inlineStr"/>
-      <c r="R72" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11891/</t>
-        </is>
-      </c>
+      <c r="R72" s="13" t="inlineStr"/>
       <c r="S72" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4322,11 +4258,7 @@
       <c r="O73" s="14" t="n"/>
       <c r="P73" s="14" t="n"/>
       <c r="Q73" s="13" t="inlineStr"/>
-      <c r="R73" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12592/</t>
-        </is>
-      </c>
+      <c r="R73" s="13" t="inlineStr"/>
       <c r="S73" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4366,11 +4298,7 @@
       <c r="O74" s="14" t="n"/>
       <c r="P74" s="14" t="n"/>
       <c r="Q74" s="13" t="inlineStr"/>
-      <c r="R74" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/13074/</t>
-        </is>
-      </c>
+      <c r="R74" s="13" t="inlineStr"/>
       <c r="S74" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4410,11 +4338,7 @@
       <c r="O75" s="14" t="n"/>
       <c r="P75" s="14" t="n"/>
       <c r="Q75" s="13" t="inlineStr"/>
-      <c r="R75" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/16651/</t>
-        </is>
-      </c>
+      <c r="R75" s="13" t="inlineStr"/>
       <c r="S75" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4550,11 +4474,7 @@
       <c r="O78" s="14" t="n"/>
       <c r="P78" s="14" t="n"/>
       <c r="Q78" s="13" t="inlineStr"/>
-      <c r="R78" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12027/</t>
-        </is>
-      </c>
+      <c r="R78" s="13" t="inlineStr"/>
       <c r="S78" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4594,11 +4514,7 @@
       <c r="O79" s="14" t="n"/>
       <c r="P79" s="14" t="n"/>
       <c r="Q79" s="13" t="inlineStr"/>
-      <c r="R79" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12520/</t>
-        </is>
-      </c>
+      <c r="R79" s="13" t="inlineStr"/>
       <c r="S79" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4640,7 +4556,7 @@
       <c r="Q80" s="13" t="inlineStr"/>
       <c r="R80" s="13" t="inlineStr">
         <is>
-          <t>[оценка] костюм антипорезный утепл. (бензопильщика) 9–14 тыс. ₽ (energocontract.ru/catalog/chain-saw — цены по запросу)</t>
+          <t>[оценка] костюм антипорезный утепл. (бензопильщика) 9–14 тыс. ₽ (energocontract.ru/ca…</t>
         </is>
       </c>
       <c r="S80" s="13" t="inlineStr">
@@ -4682,11 +4598,7 @@
       <c r="O81" s="14" t="n"/>
       <c r="P81" s="14" t="n"/>
       <c r="Q81" s="13" t="inlineStr"/>
-      <c r="R81" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11812/</t>
-        </is>
-      </c>
+      <c r="R81" s="13" t="inlineStr"/>
       <c r="S81" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4728,7 +4640,7 @@
       <c r="Q82" s="13" t="inlineStr"/>
       <c r="R82" s="13" t="inlineStr">
         <is>
-          <t>https://www.trakt.ru/catalog/zashhita-ruk/kozhanye-perchatki/ (краги РУССКИЕ ЛЬВЫ утепл.)</t>
+          <t>краги РУССКИЕ ЛЬВЫ утепл.</t>
         </is>
       </c>
       <c r="S82" s="16" t="inlineStr">
@@ -4814,11 +4726,7 @@
       <c r="O84" s="14" t="n"/>
       <c r="P84" s="14" t="n"/>
       <c r="Q84" s="13" t="inlineStr"/>
-      <c r="R84" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12001/</t>
-        </is>
-      </c>
+      <c r="R84" s="13" t="inlineStr"/>
       <c r="S84" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -4858,11 +4766,7 @@
       <c r="O85" s="14" t="n"/>
       <c r="P85" s="14" t="n"/>
       <c r="Q85" s="13" t="inlineStr"/>
-      <c r="R85" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12913/</t>
-        </is>
-      </c>
+      <c r="R85" s="13" t="inlineStr"/>
       <c r="S85" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5034,11 +4938,7 @@
       <c r="O89" s="14" t="n"/>
       <c r="P89" s="14" t="n"/>
       <c r="Q89" s="13" t="inlineStr"/>
-      <c r="R89" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11708/</t>
-        </is>
-      </c>
+      <c r="R89" s="13" t="inlineStr"/>
       <c r="S89" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5078,11 +4978,7 @@
       <c r="O90" s="14" t="n"/>
       <c r="P90" s="14" t="n"/>
       <c r="Q90" s="13" t="inlineStr"/>
-      <c r="R90" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11707/</t>
-        </is>
-      </c>
+      <c r="R90" s="13" t="inlineStr"/>
       <c r="S90" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5166,11 +5062,7 @@
       <c r="O92" s="14" t="n"/>
       <c r="P92" s="14" t="n"/>
       <c r="Q92" s="13" t="inlineStr"/>
-      <c r="R92" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/13005/</t>
-        </is>
-      </c>
+      <c r="R92" s="13" t="inlineStr"/>
       <c r="S92" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5210,11 +5102,7 @@
       <c r="O93" s="14" t="n"/>
       <c r="P93" s="14" t="n"/>
       <c r="Q93" s="13" t="inlineStr"/>
-      <c r="R93" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61033/</t>
-        </is>
-      </c>
+      <c r="R93" s="13" t="inlineStr"/>
       <c r="S93" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5298,11 +5186,7 @@
       <c r="O95" s="14" t="n"/>
       <c r="P95" s="14" t="n"/>
       <c r="Q95" s="13" t="inlineStr"/>
-      <c r="R95" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/11961/</t>
-        </is>
-      </c>
+      <c r="R95" s="13" t="inlineStr"/>
       <c r="S95" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5342,11 +5226,7 @@
       <c r="O96" s="14" t="n"/>
       <c r="P96" s="14" t="n"/>
       <c r="Q96" s="13" t="inlineStr"/>
-      <c r="R96" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61033/</t>
-        </is>
-      </c>
+      <c r="R96" s="13" t="inlineStr"/>
       <c r="S96" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5386,11 +5266,7 @@
       <c r="O97" s="14" t="n"/>
       <c r="P97" s="14" t="n"/>
       <c r="Q97" s="13" t="inlineStr"/>
-      <c r="R97" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12190/</t>
-        </is>
-      </c>
+      <c r="R97" s="13" t="inlineStr"/>
       <c r="S97" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5430,11 +5306,7 @@
       <c r="O98" s="14" t="n"/>
       <c r="P98" s="14" t="n"/>
       <c r="Q98" s="13" t="inlineStr"/>
-      <c r="R98" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/13076/</t>
-        </is>
-      </c>
+      <c r="R98" s="13" t="inlineStr"/>
       <c r="S98" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5474,11 +5346,7 @@
       <c r="O99" s="14" t="n"/>
       <c r="P99" s="14" t="n"/>
       <c r="Q99" s="13" t="inlineStr"/>
-      <c r="R99" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/61013/</t>
-        </is>
-      </c>
+      <c r="R99" s="13" t="inlineStr"/>
       <c r="S99" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5518,11 +5386,7 @@
       <c r="O100" s="14" t="n"/>
       <c r="P100" s="14" t="n"/>
       <c r="Q100" s="13" t="inlineStr"/>
-      <c r="R100" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/16450/</t>
-        </is>
-      </c>
+      <c r="R100" s="13" t="inlineStr"/>
       <c r="S100" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5562,11 +5426,7 @@
       <c r="O101" s="14" t="n"/>
       <c r="P101" s="14" t="n"/>
       <c r="Q101" s="13" t="inlineStr"/>
-      <c r="R101" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/12193/</t>
-        </is>
-      </c>
+      <c r="R101" s="13" t="inlineStr"/>
       <c r="S101" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5606,11 +5466,7 @@
       <c r="O102" s="14" t="n"/>
       <c r="P102" s="14" t="n"/>
       <c r="Q102" s="13" t="inlineStr"/>
-      <c r="R102" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/16585/</t>
-        </is>
-      </c>
+      <c r="R102" s="13" t="inlineStr"/>
       <c r="S102" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5650,11 +5506,7 @@
       <c r="O103" s="14" t="n"/>
       <c r="P103" s="14" t="n"/>
       <c r="Q103" s="13" t="inlineStr"/>
-      <c r="R103" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/product/13084/</t>
-        </is>
-      </c>
+      <c r="R103" s="13" t="inlineStr"/>
       <c r="S103" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>
@@ -5694,11 +5546,7 @@
       <c r="O104" s="14" t="n"/>
       <c r="P104" s="14" t="n"/>
       <c r="Q104" s="13" t="inlineStr"/>
-      <c r="R104" s="13" t="inlineStr">
-        <is>
-          <t>https://www.trakt.ru/catalog/specobuv/valenki/12196/</t>
-        </is>
-      </c>
+      <c r="R104" s="13" t="inlineStr"/>
       <c r="S104" s="16" t="inlineStr">
         <is>
           <t>trakt.ru</t>

</xml_diff>